<commit_message>
Updated logical data map
</commit_message>
<xml_diff>
--- a/Logical Data Map.xlsx
+++ b/Logical Data Map.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lukas\Documents\Programming\data-warehouse-project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A354ADD-5F07-494B-A6BC-3AE2705AAA5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{306E2721-6F68-4AF9-A931-F02A66958512}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{1A0EA0AD-33CE-4201-AD7F-6CC7DE1354BD}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="57">
   <si>
     <t>Mapping Change Date</t>
   </si>
@@ -153,6 +153,60 @@
   </si>
   <si>
     <t>Date</t>
+  </si>
+  <si>
+    <t>bookings</t>
+  </si>
+  <si>
+    <t>Passenger ID</t>
+  </si>
+  <si>
+    <t>First Name</t>
+  </si>
+  <si>
+    <t>Last Name</t>
+  </si>
+  <si>
+    <t>Arrival Airport</t>
+  </si>
+  <si>
+    <t>Airport Name</t>
+  </si>
+  <si>
+    <t>airports</t>
+  </si>
+  <si>
+    <t>municipality</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>iso_region</t>
+  </si>
+  <si>
+    <t>Country Name</t>
+  </si>
+  <si>
+    <t>Airport Continent</t>
+  </si>
+  <si>
+    <t>latitude_deg</t>
+  </si>
+  <si>
+    <t>longitude_deg</t>
+  </si>
+  <si>
+    <t>elevation_ft</t>
+  </si>
+  <si>
+    <t>Pilot Name</t>
+  </si>
+  <si>
+    <t>Flight Status</t>
+  </si>
+  <si>
+    <t>Departure Date</t>
   </si>
 </sst>
 </file>
@@ -247,28 +301,32 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="2"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="2" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="2" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="2"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Input" xfId="1" builtinId="20"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Output" xfId="2" builtinId="21"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -284,11 +342,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -648,50 +706,50 @@
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -708,6 +766,12 @@
       <c r="E3" t="s">
         <v>21</v>
       </c>
+      <c r="G3" t="s">
+        <v>39</v>
+      </c>
+      <c r="H3" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
@@ -719,6 +783,12 @@
       <c r="E4" t="s">
         <v>20</v>
       </c>
+      <c r="G4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H4" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
@@ -730,6 +800,12 @@
       <c r="E5" t="s">
         <v>20</v>
       </c>
+      <c r="G5" t="s">
+        <v>39</v>
+      </c>
+      <c r="H5" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
@@ -741,6 +817,12 @@
       <c r="E6" t="s">
         <v>20</v>
       </c>
+      <c r="G6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H6" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
@@ -752,6 +834,12 @@
       <c r="E7" t="s">
         <v>20</v>
       </c>
+      <c r="G7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H7" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
@@ -763,6 +851,12 @@
       <c r="E8" t="s">
         <v>20</v>
       </c>
+      <c r="G8" t="s">
+        <v>39</v>
+      </c>
+      <c r="H8" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
@@ -777,6 +871,12 @@
       <c r="E9" t="s">
         <v>21</v>
       </c>
+      <c r="G9" t="s">
+        <v>39</v>
+      </c>
+      <c r="H9" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
@@ -788,6 +888,12 @@
       <c r="E10" t="s">
         <v>20</v>
       </c>
+      <c r="G10" t="s">
+        <v>39</v>
+      </c>
+      <c r="H10" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
@@ -799,6 +905,12 @@
       <c r="E11" t="s">
         <v>20</v>
       </c>
+      <c r="G11" t="s">
+        <v>45</v>
+      </c>
+      <c r="H11" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
@@ -810,6 +922,12 @@
       <c r="E12" t="s">
         <v>20</v>
       </c>
+      <c r="G12" t="s">
+        <v>45</v>
+      </c>
+      <c r="H12" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
@@ -821,6 +939,12 @@
       <c r="E13" t="s">
         <v>20</v>
       </c>
+      <c r="G13" t="s">
+        <v>39</v>
+      </c>
+      <c r="H13" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
@@ -832,6 +956,12 @@
       <c r="E14" t="s">
         <v>20</v>
       </c>
+      <c r="G14" t="s">
+        <v>39</v>
+      </c>
+      <c r="H14" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
@@ -843,6 +973,12 @@
       <c r="E15" t="s">
         <v>20</v>
       </c>
+      <c r="G15" t="s">
+        <v>45</v>
+      </c>
+      <c r="H15" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C16" t="s">
@@ -854,8 +990,14 @@
       <c r="E16" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G16" t="s">
+        <v>45</v>
+      </c>
+      <c r="H16" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C17" t="s">
         <v>31</v>
       </c>
@@ -865,8 +1007,14 @@
       <c r="E17" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G17" t="s">
+        <v>45</v>
+      </c>
+      <c r="H17" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C18" t="s">
         <v>32</v>
       </c>
@@ -876,8 +1024,14 @@
       <c r="E18" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G18" t="s">
+        <v>45</v>
+      </c>
+      <c r="H18" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>33</v>
       </c>
@@ -891,7 +1045,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
         <v>15</v>
       </c>
@@ -901,8 +1055,14 @@
       <c r="E20" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G20" t="s">
+        <v>39</v>
+      </c>
+      <c r="H20" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C21" t="s">
         <v>16</v>
       </c>
@@ -912,8 +1072,14 @@
       <c r="E21" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G21" t="s">
+        <v>39</v>
+      </c>
+      <c r="H21" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>35</v>
       </c>
@@ -927,7 +1093,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C23" t="s">
         <v>14</v>
       </c>
@@ -937,8 +1103,14 @@
       <c r="E23" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G23" t="s">
+        <v>39</v>
+      </c>
+      <c r="H23" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C24" t="s">
         <v>23</v>
       </c>
@@ -948,8 +1120,14 @@
       <c r="E24" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G24" t="s">
+        <v>39</v>
+      </c>
+      <c r="H24" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C25" t="s">
         <v>34</v>
       </c>
@@ -960,7 +1138,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C26" t="s">
         <v>37</v>
       </c>
@@ -970,8 +1148,14 @@
       <c r="E26" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G26" t="s">
+        <v>39</v>
+      </c>
+      <c r="H26" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C27" t="s">
         <v>38</v>
       </c>
@@ -980,6 +1164,12 @@
       </c>
       <c r="E27" t="s">
         <v>20</v>
+      </c>
+      <c r="G27" t="s">
+        <v>39</v>
+      </c>
+      <c r="H27" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -988,15 +1178,22 @@
     <mergeCell ref="G1:L1"/>
   </mergeCells>
   <conditionalFormatting sqref="D1:E1048576">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="5" operator="equal">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D1:E1048576">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
-      <formula>"Yes"</formula>
+  <conditionalFormatting sqref="G1:G1048576">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+      <formula>"airports"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+      <formula>"bookings"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>